<commit_message>
docs(tracker): refresh gap rows G04, G05, G11, G15 and G16
Auto exposure and volumetric fog are in review (#397, #399), tone gates
ship (PRD-341), GPU-driven culling and projected-size culling are
partial (PRD-386, PRD-390). Cells edited in the sheet XML so the
workbook keeps its conditional formatting.
</commit_message>
<xml_diff>
--- a/docs/unreal-engine/ThreeNative_Unreal_Visual_Gap_Tracker.xlsx
+++ b/docs/unreal-engine/ThreeNative_Unreal_Visual_Gap_Tracker.xlsx
@@ -2209,17 +2209,23 @@
       <x:c r="C8" s="38" t="str">
         <x:v>Histogram-based eye adaptation and physically coherent exposure across very different scene brightness.</x:v>
       </x:c>
-      <x:c r="D8" s="38" t="str">
-        <x:v>Fixed exposure is still the default; no adaptive exposure pipeline is shipped.</x:v>
+      <x:c r="D8" s="38" t="inlineStr">
+        <x:is>
+          <x:t>Authored auto exposure and eye adaptation are implemented on PR #397 (prd:100%, open, awaiting merge); develop still ships fixed exposure. Tone measurement (PRD-341) is done.</x:t>
+        </x:is>
       </x:c>
       <x:c r="E8" s="38" t="str">
         <x:v>PRD-339; PRD-341</x:v>
       </x:c>
-      <x:c r="F8" s="38" t="str">
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="G8" s="38" t="str">
-        <x:v>PROPOSED</x:v>
+      <x:c r="F8" s="38" t="inlineStr">
+        <x:is>
+          <x:t>Partial</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G8" s="38" t="inlineStr">
+        <x:is>
+          <x:t>IN REVIEW (PR #397)</x:t>
+        </x:is>
       </x:c>
       <x:c r="H8" s="38" t="str">
         <x:v>P0</x:v>
@@ -2233,8 +2239,8 @@
       <x:c r="K8" s="38" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="L8" s="39" t="n">
-        <x:v>0</x:v>
+      <x:c r="L8" s="39">
+        <x:v>0.8</x:v>
       </x:c>
       <x:c r="M8" s="38" t="n">
         <x:f>IF(H8="P0",4,IF(H8="P1",3,IF(H8="P2",2,1)))*I8*J8</x:f>
@@ -2250,8 +2256,10 @@
       <x:c r="P8" s="38" t="str">
         <x:v>Camera Pipeline</x:v>
       </x:c>
-      <x:c r="Q8" s="38" t="str">
-        <x:v>Land PRD-341 tone measurement first, then PRD-339 exposure adaptation.</x:v>
+      <x:c r="Q8" s="38" t="inlineStr">
+        <x:is>
+          <x:t>Merge PR #397 after its template visual A/B (runbook row C1), then confirm the 10-stop settle on develop.</x:t>
+        </x:is>
       </x:c>
       <x:c r="R8" s="38" t="str">
         <x:v>Bad luminance metric or slow adaptation can make exposure intermittently wrong.</x:v>
@@ -2259,11 +2267,13 @@
       <x:c r="S8" s="38" t="str">
         <x:v>10-stop scene changes remain readable with bounded settle time and no clipping/black crush regression.</x:v>
       </x:c>
-      <x:c r="T8" s="38" t="str">
-        <x:v>https://github.com/ThreeNativeHQ/threenative/blob/main/docs/PRDs/AAA-visuals/PRD-339-the-frame-sets-its-own-exposure.md</x:v>
-      </x:c>
-      <x:c r="U8" s="41" t="n">
-        <x:v>46297</x:v>
+      <x:c r="T8" s="38" t="inlineStr">
+        <x:is>
+          <x:t>https://github.com/ThreeNativeHQ/threenative/blob/main/docs/PRDs/rendering/PRD-339-the-frame-sets-its-own-exposure.md</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="U8" s="41">
+        <x:v>46298</x:v>
       </x:c>
       <x:c r="V8" s="38" t="str">
         <x:v>The PRD itself calls this the largest look difference between a Three.js scene and a shipped game.</x:v>
@@ -2279,17 +2289,23 @@
       <x:c r="C9" s="38" t="str">
         <x:v>Production engine look is protected by automated image/tone tests and reference captures.</x:v>
       </x:c>
-      <x:c r="D9" s="38" t="str">
-        <x:v>Basic capture statistics exist, but the richer tone assertion/gate is still proposed.</x:v>
+      <x:c r="D9" s="38" t="inlineStr">
+        <x:is>
+          <x:t>assert.tone ships (PRD-341 done); world-scale gate pnpm visuals:world (same-pose + pop series, blind judges) merged in #390, its own red/green on a known-bad build pending (PRD-477 Phase 1).</x:t>
+        </x:is>
       </x:c>
       <x:c r="E9" s="38" t="str">
         <x:v>PRD-341</x:v>
       </x:c>
-      <x:c r="F9" s="38" t="str">
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="G9" s="38" t="str">
-        <x:v>PROPOSED</x:v>
+      <x:c r="F9" s="38" t="inlineStr">
+        <x:is>
+          <x:t>Partial</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G9" s="38" t="inlineStr">
+        <x:is>
+          <x:t>PRD-341 DONE; PRD-477 P1 open</x:t>
+        </x:is>
       </x:c>
       <x:c r="H9" s="38" t="str">
         <x:v>P0</x:v>
@@ -2303,8 +2319,8 @@
       <x:c r="K9" s="38" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="L9" s="39" t="n">
-        <x:v>0</x:v>
+      <x:c r="L9" s="39">
+        <x:v>0.7</x:v>
       </x:c>
       <x:c r="M9" s="38" t="n">
         <x:f>IF(H9="P0",4,IF(H9="P1",3,IF(H9="P2",2,1)))*I9*J9</x:f>
@@ -2320,8 +2336,10 @@
       <x:c r="P9" s="38" t="str">
         <x:v>Quality Gates</x:v>
       </x:c>
-      <x:c r="Q9" s="38" t="str">
-        <x:v>Implement assert.tone (mean, p1, p50, p99, clip%, black%) and wire it into visual PRDs.</x:v>
+      <x:c r="Q9" s="38" t="inlineStr">
+        <x:is>
+          <x:t>Red/green the world gate on the impostors-on build (runbook row A2), then require it on every world change.</x:t>
+        </x:is>
       </x:c>
       <x:c r="R9" s="38" t="str">
         <x:v>Without numeric gates, later rendering work can regress while screenshots still look subjectively acceptable.</x:v>
@@ -2329,11 +2347,13 @@
       <x:c r="S9" s="38" t="str">
         <x:v>AAA-look PRDs fail closed on measurable tone regressions; before/after evidence is reproducible.</x:v>
       </x:c>
-      <x:c r="T9" s="38" t="str">
-        <x:v>https://github.com/ThreeNativeHQ/threenative/blob/main/docs/PRDs/AAA-visuals/PRD-341-a-frames-tone-is-a-number-and-the-number-is-a-gate.md</x:v>
-      </x:c>
-      <x:c r="U9" s="41" t="n">
-        <x:v>46297</x:v>
+      <x:c r="T9" s="38" t="inlineStr">
+        <x:is>
+          <x:t>https://github.com/ThreeNativeHQ/threenative/blob/main/docs/PRDs/done/PRD-341-a-frames-tone-is-a-number-and-the-number-is-a-gate.md</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="U9" s="41">
+        <x:v>46298</x:v>
       </x:c>
       <x:c r="V9" s="38" t="str">
         <x:v>This is enabling infrastructure for most visual work.</x:v>
@@ -2695,17 +2715,25 @@
       <x:c r="C15" s="38" t="str">
         <x:v>Volumetric fog/clouds participate in lighting, atmosphere, depth, exposure and temporal reconstruction as one environment stack.</x:v>
       </x:c>
-      <x:c r="D15" s="38" t="str">
-        <x:v>Atmosphere foundations exist, but there is no single UE-like coherent default volumetric environment stack tracked here.</x:v>
-      </x:c>
-      <x:c r="E15" s="38" t="str">
-        <x:v>TBD (related: PRD-248)</x:v>
-      </x:c>
-      <x:c r="F15" s="38" t="str">
-        <x:v>Needs PRD</x:v>
-      </x:c>
-      <x:c r="G15" s="38" t="str">
-        <x:v>TBD</x:v>
+      <x:c r="D15" s="38" t="inlineStr">
+        <x:is>
+          <x:t>Bounded depth-correct volumetric fog is implemented on PR #399 (prd:100%, open, awaiting merge); cloud integration is not.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E15" s="38" t="inlineStr">
+        <x:is>
+          <x:t>PRD-VQ-07 (related: PRD-248)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F15" s="38" t="inlineStr">
+        <x:is>
+          <x:t>Partial</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G15" s="38" t="inlineStr">
+        <x:is>
+          <x:t>IN REVIEW (PR #399)</x:t>
+        </x:is>
       </x:c>
       <x:c r="H15" s="38" t="str">
         <x:v>P1</x:v>
@@ -2719,8 +2747,8 @@
       <x:c r="K15" s="38" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="L15" s="39" t="n">
-        <x:v>0.2</x:v>
+      <x:c r="L15" s="39">
+        <x:v>0.4</x:v>
       </x:c>
       <x:c r="M15" s="38" t="n">
         <x:f>IF(H15="P0",4,IF(H15="P1",3,IF(H15="P2",2,1)))*I15*J15</x:f>
@@ -2736,8 +2764,10 @@
       <x:c r="P15" s="38" t="str">
         <x:v>Environment</x:v>
       </x:c>
-      <x:c r="Q15" s="38" t="str">
-        <x:v>Write one scoped PRD for volumetric fog/cloud composition, temporal stability, lighting participation and native parity.</x:v>
+      <x:c r="Q15" s="38" t="inlineStr">
+        <x:is>
+          <x:t>Merge PR #399, then scope cloud composition and native parity on top of VQ-07.</x:t>
+        </x:is>
       </x:c>
       <x:c r="R15" s="38" t="str">
         <x:v>Large GPU cost and ordering interactions with GI, exposure and temporal reconstruction.</x:v>
@@ -2745,11 +2775,13 @@
       <x:c r="S15" s="38" t="str">
         <x:v>Volumetrics are stable in motion, light-aware, quality-tiered and native-parity with bounded GPU p95.</x:v>
       </x:c>
-      <x:c r="T15" s="38" t="str">
-        <x:v>https://github.com/ThreeNativeHQ/threenative/blob/main/docs/PRDs/done/PRD-248-the-atmosphere-is-luts-the-sky-is-the-games.md</x:v>
-      </x:c>
-      <x:c r="U15" s="41" t="n">
-        <x:v>46297</x:v>
+      <x:c r="T15" s="38" t="inlineStr">
+        <x:is>
+          <x:t>https://github.com/ThreeNativeHQ/threenative/blob/main/docs/PRDs/rendering/PRD-VQ-07-volumetric-fog.md</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="U15" s="41">
+        <x:v>46298</x:v>
       </x:c>
       <x:c r="V15" s="38" t="str">
         <x:v>Deliberately tracked as a gap even without a dedicated PRD.</x:v>
@@ -2973,17 +3005,23 @@
       <x:c r="C19" s="38" t="str">
         <x:v>Modern AAA renderers move visibility and submission work to the GPU to sustain dense scenes with low CPU draw overhead.</x:v>
       </x:c>
-      <x:c r="D19" s="38" t="str">
-        <x:v>Current CPU render walk has measured per-draw overhead; compute culling/indirect draw PRD is specification-only.</x:v>
+      <x:c r="D19" s="38" t="inlineStr">
+        <x:is>
+          <x:t>GPU scene compute culling and indirect draws ship for streamed worlds (PRD-473 Phase 1, #375); PRD-386's own mobile/native/per-material gates are open.</x:t>
+        </x:is>
       </x:c>
       <x:c r="E19" s="38" t="str">
         <x:v>PRD-386</x:v>
       </x:c>
-      <x:c r="F19" s="38" t="str">
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="G19" s="38" t="str">
-        <x:v>NOT STARTED</x:v>
+      <x:c r="F19" s="38" t="inlineStr">
+        <x:is>
+          <x:t>Partial</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G19" s="38" t="inlineStr">
+        <x:is>
+          <x:t>PARTIAL</x:t>
+        </x:is>
       </x:c>
       <x:c r="H19" s="38" t="str">
         <x:v>P1</x:v>
@@ -2997,8 +3035,8 @@
       <x:c r="K19" s="38" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="L19" s="39" t="n">
-        <x:v>0</x:v>
+      <x:c r="L19" s="39">
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="M19" s="38" t="n">
         <x:f>IF(H19="P0",4,IF(H19="P1",3,IF(H19="P2",2,1)))*I19*J19</x:f>
@@ -3014,8 +3052,10 @@
       <x:c r="P19" s="38" t="str">
         <x:v>Rendering Performance</x:v>
       </x:c>
-      <x:c r="Q19" s="38" t="str">
-        <x:v>Start PRD-386 when CPU draw cost is a top blocker in representative visual scenes; preserve CPU oracle/fallback.</x:v>
+      <x:c r="Q19" s="38" t="inlineStr">
+        <x:is>
+          <x:t>Close PRD-386's gates; main-pass draw cost is runbook row A4 (PRD-494).</x:t>
+        </x:is>
       </x:c>
       <x:c r="R19" s="38" t="str">
         <x:v>High cross-runtime complexity; indirect path must prove native correctness and real CPU-term reduction.</x:v>
@@ -3026,8 +3066,8 @@
       <x:c r="T19" s="38" t="str">
         <x:v>https://github.com/ThreeNativeHQ/threenative/blob/main/docs/PRDs/performance/critical/PRD-386-gpu-driven-rendering-compute-culling-and-indirect-draws.md</x:v>
       </x:c>
-      <x:c r="U19" s="41" t="n">
-        <x:v>46297</x:v>
+      <x:c r="U19" s="41">
+        <x:v>46298</x:v>
       </x:c>
       <x:c r="V19" s="38" t="str">
         <x:v>Primarily an enabler for visual density rather than a direct look feature.</x:v>
@@ -3043,17 +3083,23 @@
       <x:c r="C20" s="38" t="str">
         <x:v>Objects below resolvable pixel size are aggressively culled/LOD'd by engine-level visibility systems.</x:v>
       </x:c>
-      <x:c r="D20" s="38" t="str">
-        <x:v>Real games proved the win, but the engine-default projected-size policy PRD remains specification-only.</x:v>
+      <x:c r="D20" s="38" t="inlineStr">
+        <x:is>
+          <x:t>Render-camera projected-size culling ships (render-camera-cull, #263, 8c182343f); PRD-390's measured gates are unticked.</x:t>
+        </x:is>
       </x:c>
       <x:c r="E20" s="38" t="str">
         <x:v>PRD-390</x:v>
       </x:c>
-      <x:c r="F20" s="38" t="str">
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="G20" s="38" t="str">
-        <x:v>NOT STARTED</x:v>
+      <x:c r="F20" s="38" t="inlineStr">
+        <x:is>
+          <x:t>Partial</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G20" s="38" t="inlineStr">
+        <x:is>
+          <x:t>PARTIAL</x:t>
+        </x:is>
       </x:c>
       <x:c r="H20" s="38" t="str">
         <x:v>P1</x:v>
@@ -3067,8 +3113,8 @@
       <x:c r="K20" s="38" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L20" s="39" t="n">
-        <x:v>0.1</x:v>
+      <x:c r="L20" s="39">
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="M20" s="38" t="n">
         <x:f>IF(H20="P0",4,IF(H20="P1",3,IF(H20="P2",2,1)))*I20*J20</x:f>
@@ -3084,8 +3130,10 @@
       <x:c r="P20" s="38" t="str">
         <x:v>Rendering Performance</x:v>
       </x:c>
-      <x:c r="Q20" s="38" t="str">
-        <x:v>Execute conservative projected-size default with a pixel-diff ladder and explicit opt-out.</x:v>
+      <x:c r="Q20" s="38" t="inlineStr">
+        <x:is>
+          <x:t>Tick PRD-390's gates with the pixel-diff ladder on a representative scene.</x:t>
+        </x:is>
       </x:c>
       <x:c r="R20" s="38" t="str">
         <x:v>Default changes what every game draws; must prove image equivalence at ordinary player views.</x:v>
@@ -3096,8 +3144,8 @@
       <x:c r="T20" s="38" t="str">
         <x:v>https://github.com/ThreeNativeHQ/threenative/blob/main/docs/PRDs/performance/critical/PRD-390-do-not-submit-what-the-render-camera-cannot-resolve.md</x:v>
       </x:c>
-      <x:c r="U20" s="41" t="n">
-        <x:v>46297</x:v>
+      <x:c r="U20" s="41">
+        <x:v>46298</x:v>
       </x:c>
       <x:c r="V20" s="38" t="str"/>
     </x:row>

</xml_diff>